<commit_message>
avances hasta la celda del video de ski en la montaña
</commit_message>
<xml_diff>
--- a/Lab_4/src/validation_set_results.xlsx
+++ b/Lab_4/src/validation_set_results.xlsx
@@ -518,43 +518,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J2" t="n">
         <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G2" t="n">
-        <v>10</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>30</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
       </c>
       <c r="K2" t="n">
         <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -573,13 +573,13 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -591,25 +591,25 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>1</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
@@ -628,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -646,22 +646,22 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -674,49 +674,49 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
         <v>2</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>4</v>
       </c>
       <c r="O5" t="n">
         <v>4</v>
       </c>
       <c r="P5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
@@ -735,40 +735,40 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
         <v>32</v>
       </c>
       <c r="G6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
         <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="O6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -778,19 +778,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G7" t="n">
         <v>55</v>
@@ -799,28 +799,28 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C8" t="n">
         <v>1</v>
@@ -839,40 +839,40 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H8" t="n">
         <v>6</v>
       </c>
       <c r="I8" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" t="n">
         <v>2</v>
       </c>
       <c r="P8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -882,10 +882,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -894,37 +894,37 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O9" t="n">
         <v>2</v>
       </c>
       <c r="P9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -937,13 +937,13 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -958,22 +958,22 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -995,40 +995,40 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
+        <v>22</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>28</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
         <v>20</v>
-      </c>
-      <c r="H11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" t="n">
-        <v>32</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>23</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1038,19 +1038,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D12" t="n">
         <v>7</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -1059,25 +1059,25 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>17</v>
+      </c>
+      <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="n">
-        <v>15</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1</v>
-      </c>
       <c r="L12" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1093,43 +1093,43 @@
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G13" t="n">
         <v>7</v>
       </c>
       <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
         <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>5</v>
-      </c>
-      <c r="J13" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
@@ -1145,7 +1145,7 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -1154,19 +1154,19 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
         <v>4</v>
-      </c>
-      <c r="J14" t="n">
-        <v>2</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1178,13 +1178,13 @@
         <v>7</v>
       </c>
       <c r="N14" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -1224,16 +1224,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="P15" t="n">
         <v>1</v>
@@ -1249,25 +1249,25 @@
         <v>0</v>
       </c>
       <c r="C16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" t="n">
-        <v>3</v>
-      </c>
       <c r="G16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
@@ -1276,19 +1276,19 @@
         <v>1</v>
       </c>
       <c r="L16" t="n">
+        <v>6</v>
+      </c>
+      <c r="M16" t="n">
         <v>3</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>2</v>
       </c>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
       <c r="O16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P16" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2899,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -4225,7 +4225,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -4718,7 +4718,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -5517,7 +5517,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -6554,7 +6554,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -6673,7 +6673,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -6877,7 +6877,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -6894,7 +6894,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -6996,7 +6996,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -7234,7 +7234,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -7285,7 +7285,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7302,7 +7302,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -7387,7 +7387,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -7404,7 +7404,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7421,7 +7421,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7489,7 +7489,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -7693,7 +7693,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7727,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -7846,7 +7846,7 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7897,7 +7897,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -7931,7 +7931,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -7948,7 +7948,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -8084,7 +8084,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8101,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -8135,7 +8135,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -8169,7 +8169,7 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -8203,7 +8203,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -8237,7 +8237,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -8475,7 +8475,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -8526,7 +8526,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -8577,7 +8577,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -8713,7 +8713,7 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -8730,7 +8730,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -8747,7 +8747,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8832,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -8849,7 +8849,7 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -8900,7 +8900,7 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -8934,7 +8934,7 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9121,7 +9121,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9189,7 +9189,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -9206,7 +9206,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -9342,7 +9342,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -9410,7 +9410,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9427,7 +9427,7 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9495,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9631,7 +9631,7 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -9716,7 +9716,7 @@
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -9784,7 +9784,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -9869,7 +9869,7 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -10005,7 +10005,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -10022,7 +10022,7 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -10073,7 +10073,7 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -10243,7 +10243,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -10345,7 +10345,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -10413,7 +10413,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -10430,7 +10430,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -10498,7 +10498,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -10515,7 +10515,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -10532,7 +10532,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -10600,7 +10600,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -10617,7 +10617,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -10634,7 +10634,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -10770,7 +10770,7 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -10923,7 +10923,7 @@
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -11008,7 +11008,7 @@
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -11025,7 +11025,7 @@
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -11059,7 +11059,7 @@
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -11127,7 +11127,7 @@
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -11144,7 +11144,7 @@
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -11246,7 +11246,7 @@
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -11314,7 +11314,7 @@
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -11348,7 +11348,7 @@
       </c>
       <c r="C591" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -11569,7 +11569,7 @@
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -11586,7 +11586,7 @@
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -11603,7 +11603,7 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -11620,7 +11620,7 @@
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -11637,7 +11637,7 @@
       </c>
       <c r="C608" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -11671,7 +11671,7 @@
       </c>
       <c r="C610" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -11688,7 +11688,7 @@
       </c>
       <c r="C611" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -11756,7 +11756,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -11773,7 +11773,7 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -11807,7 +11807,7 @@
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -11858,7 +11858,7 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -11875,7 +11875,7 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -11892,7 +11892,7 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -11994,7 +11994,7 @@
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -12028,7 +12028,7 @@
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -12079,7 +12079,7 @@
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -12096,7 +12096,7 @@
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -12130,7 +12130,7 @@
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -12215,7 +12215,7 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -12334,7 +12334,7 @@
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -12402,7 +12402,7 @@
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -12436,7 +12436,7 @@
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -12470,7 +12470,7 @@
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -12504,7 +12504,7 @@
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -12521,7 +12521,7 @@
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -12674,7 +12674,7 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -12725,7 +12725,7 @@
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -12759,7 +12759,7 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -12827,7 +12827,7 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -12861,7 +12861,7 @@
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -12912,7 +12912,7 @@
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -13031,7 +13031,7 @@
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -13048,7 +13048,7 @@
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -13065,7 +13065,7 @@
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13082,7 +13082,7 @@
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -13133,7 +13133,7 @@
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -13150,7 +13150,7 @@
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -13201,7 +13201,7 @@
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -13235,7 +13235,7 @@
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13269,7 +13269,7 @@
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13286,7 +13286,7 @@
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -13320,7 +13320,7 @@
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13337,7 +13337,7 @@
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -13354,7 +13354,7 @@
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -13371,7 +13371,7 @@
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13456,7 +13456,7 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13490,7 +13490,7 @@
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13541,7 +13541,7 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -13558,7 +13558,7 @@
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -13575,7 +13575,7 @@
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -13609,7 +13609,7 @@
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -13762,7 +13762,7 @@
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13779,7 +13779,7 @@
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -13813,7 +13813,7 @@
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -13830,7 +13830,7 @@
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13847,7 +13847,7 @@
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -13881,7 +13881,7 @@
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13898,7 +13898,7 @@
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -13915,7 +13915,7 @@
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14000,7 +14000,7 @@
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -14153,7 +14153,7 @@
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14272,7 +14272,7 @@
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14289,7 +14289,7 @@
       </c>
       <c r="C764" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -14357,7 +14357,7 @@
       </c>
       <c r="C768" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -14391,7 +14391,7 @@
       </c>
       <c r="C770" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -14425,7 +14425,7 @@
       </c>
       <c r="C772" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14459,7 +14459,7 @@
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14544,7 +14544,7 @@
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -14629,7 +14629,7 @@
       </c>
       <c r="C784" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -14646,7 +14646,7 @@
       </c>
       <c r="C785" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -14663,7 +14663,7 @@
       </c>
       <c r="C786" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -14714,7 +14714,7 @@
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -14765,7 +14765,7 @@
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>Bedroom</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -14782,7 +14782,7 @@
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -14816,7 +14816,7 @@
       </c>
       <c r="C795" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -14867,7 +14867,7 @@
       </c>
       <c r="C798" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -14884,7 +14884,7 @@
       </c>
       <c r="C799" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -14901,7 +14901,7 @@
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -15054,7 +15054,7 @@
       </c>
       <c r="C809" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -15088,7 +15088,7 @@
       </c>
       <c r="C811" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -15190,7 +15190,7 @@
       </c>
       <c r="C817" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -15241,7 +15241,7 @@
       </c>
       <c r="C820" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -15258,7 +15258,7 @@
       </c>
       <c r="C821" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -15275,7 +15275,7 @@
       </c>
       <c r="C822" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -15343,7 +15343,7 @@
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="C827" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -15394,7 +15394,7 @@
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -15496,7 +15496,7 @@
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -15513,7 +15513,7 @@
       </c>
       <c r="C836" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -15632,7 +15632,7 @@
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -15785,7 +15785,7 @@
       </c>
       <c r="C852" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -15819,7 +15819,7 @@
       </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -15955,7 +15955,7 @@
       </c>
       <c r="C862" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -15972,7 +15972,7 @@
       </c>
       <c r="C863" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -16006,7 +16006,7 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -16193,7 +16193,7 @@
       </c>
       <c r="C876" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16210,7 +16210,7 @@
       </c>
       <c r="C877" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16312,7 @@
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16346,7 +16346,7 @@
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16363,7 +16363,7 @@
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16482,7 +16482,7 @@
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16533,7 +16533,7 @@
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -16601,7 +16601,7 @@
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -16737,7 +16737,7 @@
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -16890,7 +16890,7 @@
       </c>
       <c r="C917" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -16941,7 +16941,7 @@
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -16992,7 +16992,7 @@
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -17077,7 +17077,7 @@
       </c>
       <c r="C928" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -17111,7 +17111,7 @@
       </c>
       <c r="C930" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -17128,7 +17128,7 @@
       </c>
       <c r="C931" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -17145,7 +17145,7 @@
       </c>
       <c r="C932" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -17162,7 +17162,7 @@
       </c>
       <c r="C933" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -17230,7 +17230,7 @@
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -17332,7 +17332,7 @@
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -17349,7 +17349,7 @@
       </c>
       <c r="C944" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -17366,7 +17366,7 @@
       </c>
       <c r="C945" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -17383,7 +17383,7 @@
       </c>
       <c r="C946" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -17400,7 +17400,7 @@
       </c>
       <c r="C947" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -17434,7 +17434,7 @@
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17451,7 @@
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -17485,7 +17485,7 @@
       </c>
       <c r="C952" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -17519,7 +17519,7 @@
       </c>
       <c r="C954" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -17536,7 +17536,7 @@
       </c>
       <c r="C955" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -17672,7 +17672,7 @@
       </c>
       <c r="C963" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -17706,7 +17706,7 @@
       </c>
       <c r="C965" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -17740,7 +17740,7 @@
       </c>
       <c r="C967" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -17842,7 +17842,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -17859,7 +17859,7 @@
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -17876,7 +17876,7 @@
       </c>
       <c r="C975" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -17893,7 +17893,7 @@
       </c>
       <c r="C976" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -17927,7 +17927,7 @@
       </c>
       <c r="C978" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -18029,7 +18029,7 @@
       </c>
       <c r="C984" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -18046,7 +18046,7 @@
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -18233,7 +18233,7 @@
       </c>
       <c r="C996" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -18267,7 +18267,7 @@
       </c>
       <c r="C998" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -18301,7 +18301,7 @@
       </c>
       <c r="C1000" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -18335,7 +18335,7 @@
       </c>
       <c r="C1002" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -18352,7 +18352,7 @@
       </c>
       <c r="C1003" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18386,7 +18386,7 @@
       </c>
       <c r="C1005" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18454,7 +18454,7 @@
       </c>
       <c r="C1009" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -18505,7 +18505,7 @@
       </c>
       <c r="C1012" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -18522,7 +18522,7 @@
       </c>
       <c r="C1013" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18556,7 +18556,7 @@
       </c>
       <c r="C1015" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18607,7 +18607,7 @@
       </c>
       <c r="C1018" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -18641,7 +18641,7 @@
       </c>
       <c r="C1020" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -18709,7 +18709,7 @@
       </c>
       <c r="C1024" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18777,7 +18777,7 @@
       </c>
       <c r="C1028" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -18794,7 +18794,7 @@
       </c>
       <c r="C1029" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -18845,7 +18845,7 @@
       </c>
       <c r="C1032" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -18896,7 +18896,7 @@
       </c>
       <c r="C1035" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -18913,7 +18913,7 @@
       </c>
       <c r="C1036" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C1038" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -18964,7 +18964,7 @@
       </c>
       <c r="C1039" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -18998,7 +18998,7 @@
       </c>
       <c r="C1041" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19015,7 +19015,7 @@
       </c>
       <c r="C1042" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -19066,7 +19066,7 @@
       </c>
       <c r="C1045" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19083,7 +19083,7 @@
       </c>
       <c r="C1046" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -19100,7 +19100,7 @@
       </c>
       <c r="C1047" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19117,7 +19117,7 @@
       </c>
       <c r="C1048" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -19168,7 +19168,7 @@
       </c>
       <c r="C1051" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -19202,7 +19202,7 @@
       </c>
       <c r="C1053" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -19236,7 +19236,7 @@
       </c>
       <c r="C1055" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -19304,7 +19304,7 @@
       </c>
       <c r="C1059" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -19406,7 +19406,7 @@
       </c>
       <c r="C1065" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19491,7 +19491,7 @@
       </c>
       <c r="C1070" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19525,7 +19525,7 @@
       </c>
       <c r="C1072" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19576,7 +19576,7 @@
       </c>
       <c r="C1075" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -19593,7 +19593,7 @@
       </c>
       <c r="C1076" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Bedroom</t>
         </is>
       </c>
     </row>
@@ -19712,7 +19712,7 @@
       </c>
       <c r="C1083" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -19831,7 +19831,7 @@
       </c>
       <c r="C1090" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -19882,7 +19882,7 @@
       </c>
       <c r="C1093" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -20001,7 +20001,7 @@
       </c>
       <c r="C1100" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -20086,7 +20086,7 @@
       </c>
       <c r="C1105" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -20154,7 +20154,7 @@
       </c>
       <c r="C1109" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -20273,7 +20273,7 @@
       </c>
       <c r="C1116" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -20443,7 +20443,7 @@
       </c>
       <c r="C1126" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -20647,7 +20647,7 @@
       </c>
       <c r="C1138" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -20681,7 +20681,7 @@
       </c>
       <c r="C1140" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -20936,7 +20936,7 @@
       </c>
       <c r="C1155" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -20970,7 +20970,7 @@
       </c>
       <c r="C1157" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -20987,7 +20987,7 @@
       </c>
       <c r="C1158" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -21055,7 +21055,7 @@
       </c>
       <c r="C1162" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C1172" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -21242,7 +21242,7 @@
       </c>
       <c r="C1173" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21259,7 +21259,7 @@
       </c>
       <c r="C1174" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21310,7 +21310,7 @@
       </c>
       <c r="C1177" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>Kitchen</t>
         </is>
       </c>
     </row>
@@ -21412,7 +21412,7 @@
       </c>
       <c r="C1183" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -21463,7 +21463,7 @@
       </c>
       <c r="C1186" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21514,7 +21514,7 @@
       </c>
       <c r="C1189" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -21599,7 +21599,7 @@
       </c>
       <c r="C1194" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -21667,7 +21667,7 @@
       </c>
       <c r="C1198" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -21752,7 +21752,7 @@
       </c>
       <c r="C1203" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="C1207" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21837,7 +21837,7 @@
       </c>
       <c r="C1208" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -21854,7 +21854,7 @@
       </c>
       <c r="C1209" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -21871,7 +21871,7 @@
       </c>
       <c r="C1210" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21888,7 +21888,7 @@
       </c>
       <c r="C1211" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -21922,7 +21922,7 @@
       </c>
       <c r="C1213" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -21956,7 +21956,7 @@
       </c>
       <c r="C1215" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -21973,7 +21973,7 @@
       </c>
       <c r="C1216" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -22007,7 +22007,7 @@
       </c>
       <c r="C1218" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -22058,7 +22058,7 @@
       </c>
       <c r="C1221" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -22075,7 +22075,7 @@
       </c>
       <c r="C1222" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22245,7 +22245,7 @@
       </c>
       <c r="C1232" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -22279,7 +22279,7 @@
       </c>
       <c r="C1234" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -22330,7 +22330,7 @@
       </c>
       <c r="C1237" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -22415,7 +22415,7 @@
       </c>
       <c r="C1242" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22432,7 +22432,7 @@
       </c>
       <c r="C1243" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -22449,7 +22449,7 @@
       </c>
       <c r="C1244" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -22483,7 +22483,7 @@
       </c>
       <c r="C1246" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22500,7 +22500,7 @@
       </c>
       <c r="C1247" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22517,7 +22517,7 @@
       </c>
       <c r="C1248" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -22534,7 +22534,7 @@
       </c>
       <c r="C1249" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -22568,7 +22568,7 @@
       </c>
       <c r="C1251" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -22670,7 +22670,7 @@
       </c>
       <c r="C1257" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22704,7 +22704,7 @@
       </c>
       <c r="C1259" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -22721,7 +22721,7 @@
       </c>
       <c r="C1260" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22755,7 +22755,7 @@
       </c>
       <c r="C1262" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -22772,7 +22772,7 @@
       </c>
       <c r="C1263" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -22789,7 +22789,7 @@
       </c>
       <c r="C1264" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -22823,7 +22823,7 @@
       </c>
       <c r="C1266" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -22908,7 +22908,7 @@
       </c>
       <c r="C1271" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22942,7 +22942,7 @@
       </c>
       <c r="C1273" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -22959,7 +22959,7 @@
       </c>
       <c r="C1274" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -23010,7 +23010,7 @@
       </c>
       <c r="C1277" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -23027,7 +23027,7 @@
       </c>
       <c r="C1278" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -23044,7 +23044,7 @@
       </c>
       <c r="C1279" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -23078,7 +23078,7 @@
       </c>
       <c r="C1281" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -23282,7 +23282,7 @@
       </c>
       <c r="C1293" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -23333,7 +23333,7 @@
       </c>
       <c r="C1296" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -23350,7 +23350,7 @@
       </c>
       <c r="C1297" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -23775,7 +23775,7 @@
       </c>
       <c r="C1322" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -23792,7 +23792,7 @@
       </c>
       <c r="C1323" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -23843,7 +23843,7 @@
       </c>
       <c r="C1326" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Forest</t>
         </is>
       </c>
     </row>
@@ -23928,7 +23928,7 @@
       </c>
       <c r="C1331" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -24047,7 +24047,7 @@
       </c>
       <c r="C1338" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -24064,7 +24064,7 @@
       </c>
       <c r="C1339" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -24217,7 +24217,7 @@
       </c>
       <c r="C1348" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -24370,7 +24370,7 @@
       </c>
       <c r="C1357" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -24506,7 +24506,7 @@
       </c>
       <c r="C1365" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -24557,7 +24557,7 @@
       </c>
       <c r="C1368" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -24676,7 +24676,7 @@
       </c>
       <c r="C1375" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -25016,7 +25016,7 @@
       </c>
       <c r="C1395" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -25084,7 +25084,7 @@
       </c>
       <c r="C1399" t="inlineStr">
         <is>
-          <t>Open country</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -25118,7 +25118,7 @@
       </c>
       <c r="C1401" t="inlineStr">
         <is>
-          <t>Suburb</t>
+          <t>Highway</t>
         </is>
       </c>
     </row>
@@ -25169,7 +25169,7 @@
       </c>
       <c r="C1404" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -25186,7 +25186,7 @@
       </c>
       <c r="C1405" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -25339,7 +25339,7 @@
       </c>
       <c r="C1414" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -25441,7 +25441,7 @@
       </c>
       <c r="C1420" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -25492,7 +25492,7 @@
       </c>
       <c r="C1423" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Mountain</t>
         </is>
       </c>
     </row>
@@ -25509,7 +25509,7 @@
       </c>
       <c r="C1424" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -25526,7 +25526,7 @@
       </c>
       <c r="C1425" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Suburb</t>
         </is>
       </c>
     </row>
@@ -25560,7 +25560,7 @@
       </c>
       <c r="C1427" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -25628,7 +25628,7 @@
       </c>
       <c r="C1431" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -25696,7 +25696,7 @@
       </c>
       <c r="C1435" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -25730,7 +25730,7 @@
       </c>
       <c r="C1437" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Living room</t>
         </is>
       </c>
     </row>
@@ -25781,7 +25781,7 @@
       </c>
       <c r="C1440" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -25866,7 +25866,7 @@
       </c>
       <c r="C1445" t="inlineStr">
         <is>
-          <t>Mountain</t>
+          <t>Store</t>
         </is>
       </c>
     </row>
@@ -25900,7 +25900,7 @@
       </c>
       <c r="C1447" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -25917,7 +25917,7 @@
       </c>
       <c r="C1448" t="inlineStr">
         <is>
-          <t>Inside city</t>
+          <t>Street</t>
         </is>
       </c>
     </row>
@@ -25985,7 +25985,7 @@
       </c>
       <c r="C1452" t="inlineStr">
         <is>
-          <t>Street</t>
+          <t>Open country</t>
         </is>
       </c>
     </row>
@@ -26053,7 +26053,7 @@
       </c>
       <c r="C1456" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -26087,7 +26087,7 @@
       </c>
       <c r="C1458" t="inlineStr">
         <is>
-          <t>Coast</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -26240,7 +26240,7 @@
       </c>
       <c r="C1467" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -26291,7 +26291,7 @@
       </c>
       <c r="C1470" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -26342,7 +26342,7 @@
       </c>
       <c r="C1473" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -26427,7 +26427,7 @@
       </c>
       <c r="C1478" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -26444,7 +26444,7 @@
       </c>
       <c r="C1479" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -26478,7 +26478,7 @@
       </c>
       <c r="C1481" t="inlineStr">
         <is>
-          <t>Living room</t>
+          <t>Tall building</t>
         </is>
       </c>
     </row>
@@ -26495,7 +26495,7 @@
       </c>
       <c r="C1482" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Inside city</t>
         </is>
       </c>
     </row>
@@ -26580,7 +26580,7 @@
       </c>
       <c r="C1487" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -26716,7 +26716,7 @@
       </c>
       <c r="C1495" t="inlineStr">
         <is>
-          <t>Tall building</t>
+          <t>Coast</t>
         </is>
       </c>
     </row>
@@ -26750,7 +26750,7 @@
       </c>
       <c r="C1497" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>

</xml_diff>